<commit_message>
I have been update something in here
</commit_message>
<xml_diff>
--- a/build/bookings.xlsx
+++ b/build/bookings.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
   <si>
     <t>BookingID</t>
   </si>
@@ -52,28 +52,55 @@
     <t>1</t>
   </si>
   <si>
-    <t>korea</t>
-  </si>
-  <si>
-    <t>student</t>
+    <t>Smey</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>250.00</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>VIP</t>
-  </si>
-  <si>
-    <t>1000.00</t>
-  </si>
-  <si>
-    <t>2026-04-26</t>
+    <t>500.00</t>
+  </si>
+  <si>
+    <t>Thanuk</t>
+  </si>
+  <si>
+    <t>Nuk</t>
+  </si>
+  <si>
+    <t>101</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>100.00</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>300.00</t>
+  </si>
+  <si>
+    <t>lyheng</t>
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>2000.00</t>
   </si>
   <si>
     <t>0</t>
@@ -386,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -432,31 +459,101 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="C3" t="s">
         <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>